<commit_message>
Update application system to navigate directly to form when data is selected
Modify the "데이터 조회" section to allow users to click on a row to automatically navigate to the "신청서 작성" menu and load the selected application data, replacing the "이 신청서 수정하기" button. Implement session state management for menu navigation and update PDF metadata creation timestamps.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 710ff447-e995-4e1a-8356-f5d3a8557502
Replit-Commit-Checkpoint-Type: intermediate_checkpoint
Replit-Commit-Event-Id: 77e35f32-a817-411e-ba2a-c153103d785a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/710ff447-e995-4e1a-8356-f5d3a8557502/eEdOlBo
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/management_db.xlsx
+++ b/management_db.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,6 +467,52 @@
         <is>
           <t>합계금액</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>최재혁</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>회색동복</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -480,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -503,6 +549,26 @@
         <is>
           <t>총액</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Make data table rows clickable for direct editing
Replace the separate query section with a selectable data table, enabling direct row editing and removing the old query interface.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 710ff447-e995-4e1a-8356-f5d3a8557502
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a642ef00-22cb-480d-8876-8841e3c0087a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/710ff447-e995-4e1a-8356-f5d3a8557502/7hVYeqR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/management_db.xlsx
+++ b/management_db.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,52 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>최재혁</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>회색동복</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix editing functionality and remove unnecessary columns from the data view
Update the UI to properly navigate to the application form when an edit button is clicked and remove the 'Total Amount' and 'Corporation' columns from the data inquiry view.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 710ff447-e995-4e1a-8356-f5d3a8557502
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: cf4e3e37-51d9-4cad-bf0e-d77e42120f24
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/710ff447-e995-4e1a-8356-f5d3a8557502/ol6DaDR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/management_db.xlsx
+++ b/management_db.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -558,6 +558,52 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>경비물품</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>최재혁</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">휴지 </t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>100M</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update application form and header to reflect company branding
Modify PDF generation to include company logo in header and update footer text.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 710ff447-e995-4e1a-8356-f5d3a8557502
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: c4fcdeef-3fe5-4473-91e5-b9f7ba492cf7
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/710ff447-e995-4e1a-8356-f5d3a8557502/k5HcOde
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/management_db.xlsx
+++ b/management_db.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -605,6 +605,52 @@
       </c>
       <c r="J4" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026. 01. 14.</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>우장산꿈에그린</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>김솔휘</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>동계상의(회색동복)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" t="n">
+        <v>19500</v>
+      </c>
+      <c r="J5" t="n">
+        <v>19500</v>
       </c>
     </row>
   </sheetData>
@@ -618,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -656,10 +702,30 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>우장산꿈에그린</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>정화빌딩</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D3" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update application form and fix errors in report generation and date handling
Modify placeholder text for remarks, correct date parsing logic in the Excel handler to prevent errors, and remove outdated draft entries.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 65b4c133-1c29-403a-a908-af2de34cc2d3
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 83bde9a4-2779-4c5c-a063-1bb240a7b46d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/af6b671c-f086-4da8-9571-39668ddf1e8b/65b4c133-1c29-403a-a908-af2de34cc2d3/D4lAwor
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/management_db.xlsx
+++ b/management_db.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -650,6 +650,236 @@
         <v>19500</v>
       </c>
       <c r="J5" t="n">
+        <v>19500</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>강용석</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>회색동복</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>강용석</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>회색동복</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>강용석</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>회색동복</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026. 01. 13.</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>정화빌딩</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>강용석</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>회색동복</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026. 01. 14.</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>피복</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>미래</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>우장산꿈에그린</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>김솔휘</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>동계상의(회색동복)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>상의:100/하의:32/모자:중</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>19500</v>
+      </c>
+      <c r="J10" t="n">
         <v>19500</v>
       </c>
     </row>
@@ -706,7 +936,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>19500</v>
+        <v>39000</v>
       </c>
     </row>
     <row r="3">

</xml_diff>